<commit_message>
Add revenue-by-segment tab to AAPL model
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Gurdev_AAPL_Financial_Model.xlsx
+++ b/models/Gurdev_AAPL_Financial_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devsingh/coursework-portfolio/models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FDFACF-F080-7E4E-BBC5-FF2E3B2FD0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58594DA0-8D82-8A4E-8D35-98FFBD4DCCA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,8 @@
     <sheet name="CashFlow" sheetId="5" r:id="rId5"/>
     <sheet name="DCF" sheetId="6" r:id="rId6"/>
     <sheet name="Comps" sheetId="7" r:id="rId7"/>
-    <sheet name="Earnings" sheetId="8" r:id="rId8"/>
+    <sheet name="SegmentRevenue" sheetId="8" r:id="rId8"/>
+    <sheet name="Earnings" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="212">
   <si>
     <t>Apple Inc. (AAPL) — Valuation Summary</t>
   </si>
@@ -544,6 +545,69 @@
   </si>
   <si>
     <t>Peer multiples: Yahoo Finance, 2026-07-18. Peer set: MSFT, GOOGL, NVDA, META (mega-cap tech).</t>
+  </si>
+  <si>
+    <t>AAPL — Revenue by Product Category ($bn)</t>
+  </si>
+  <si>
+    <t>iPhone</t>
+  </si>
+  <si>
+    <t>Mac</t>
+  </si>
+  <si>
+    <t>iPad</t>
+  </si>
+  <si>
+    <t>Wearables, Home &amp; Accessories</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Total net sales</t>
+  </si>
+  <si>
+    <t>Tie to Income Statement (must be ~0)</t>
+  </si>
+  <si>
+    <t>Revenue mix (% of total)</t>
+  </si>
+  <si>
+    <t>Growth YoY</t>
+  </si>
+  <si>
+    <t>Subscriptions — what Apple actually discloses</t>
+  </si>
+  <si>
+    <t>Apple does NOT report subscription revenue as a separate line. The closest disclosed figure is the</t>
+  </si>
+  <si>
+    <t>Services segment: $109.2bn in FY2025 (26.2% of revenue), first year above $100bn, growing ~14%/yr.</t>
+  </si>
+  <si>
+    <t>Services bundles subscriptions (iCloud, Apple Music, TV+, Arcade, News+, Fitness+, AppleCare plans,</t>
+  </si>
+  <si>
+    <t>third-party app subscriptions sold via App Store) together with App Store commissions, advertising,</t>
+  </si>
+  <si>
+    <t>and payment services - so Services revenue overstates pure subscription revenue.</t>
+  </si>
+  <si>
+    <t>Scale disclosure: Apple reports 'more than 1 billion' cumulative paid subscriptions across its</t>
+  </si>
+  <si>
+    <t>platforms (crossed in Jan 2025; more than doubled over four years).</t>
+  </si>
+  <si>
+    <t>Services carried a ~74% gross margin in recent years vs ~37% for products - the mix shift toward</t>
+  </si>
+  <si>
+    <t>Services is the main driver of total gross margin rising from 43.3% (FY22) to 46.9% (FY25).</t>
+  </si>
+  <si>
+    <t>Sources: Apple Form 10-K FY2025 (SEC EDGAR, aapl-20250927) and FY2023 10-K for FY2022 figures; Apple press disclosures for subscription counts.</t>
   </si>
   <si>
     <t>AAPL — Earnings Review</t>
@@ -620,13 +684,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="\$#,##0.0;\(\$#,##0.0\);\-"/>
-    <numFmt numFmtId="166" formatCode="\$0.00"/>
+    <numFmt numFmtId="164" formatCode="\$0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.0;\(\$#,##0.0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0\x"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -670,8 +734,38 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF808080"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -686,6 +780,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -710,38 +809,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1051,7 +1162,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1224,7 +1335,7 @@
     <col min="9" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -1701,7 +1812,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>84</v>
       </c>
@@ -2373,7 +2484,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
@@ -3001,7 +3112,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>122</v>
       </c>
@@ -3435,7 +3546,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
@@ -3808,7 +3919,7 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>148</v>
       </c>
@@ -4052,6 +4163,421 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="5" width="11.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="29" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" s="32">
+        <v>205.5</v>
+      </c>
+      <c r="C3" s="32">
+        <v>200.6</v>
+      </c>
+      <c r="D3" s="32">
+        <v>201.2</v>
+      </c>
+      <c r="E3" s="32">
+        <v>209.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="32">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="C4" s="32">
+        <v>29.4</v>
+      </c>
+      <c r="D4" s="32">
+        <v>30</v>
+      </c>
+      <c r="E4" s="32">
+        <v>33.700000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" s="32">
+        <v>29.3</v>
+      </c>
+      <c r="C5" s="32">
+        <v>28.3</v>
+      </c>
+      <c r="D5" s="32">
+        <v>26.7</v>
+      </c>
+      <c r="E5" s="32">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="31" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="32">
+        <v>41.2</v>
+      </c>
+      <c r="C6" s="32">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="D6" s="32">
+        <v>37</v>
+      </c>
+      <c r="E6" s="32">
+        <v>35.700000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" s="32">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="C7" s="32">
+        <v>85.2</v>
+      </c>
+      <c r="D7" s="32">
+        <v>96.2</v>
+      </c>
+      <c r="E7" s="32">
+        <v>109.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="34">
+        <f>SUM(B3:B7)</f>
+        <v>394.29999999999995</v>
+      </c>
+      <c r="C8" s="34">
+        <f>SUM(C3:C7)</f>
+        <v>383.3</v>
+      </c>
+      <c r="D8" s="34">
+        <f>SUM(D3:D7)</f>
+        <v>391.09999999999997</v>
+      </c>
+      <c r="E8" s="34">
+        <f>SUM(E3:E7)</f>
+        <v>416.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" s="35">
+        <f>B8-IncomeStatement!B3</f>
+        <v>-3.0000000000029559E-2</v>
+      </c>
+      <c r="C9" s="35">
+        <f>C8-IncomeStatement!C3</f>
+        <v>9.9999999999909051E-3</v>
+      </c>
+      <c r="D9" s="35">
+        <f>D8-IncomeStatement!D3</f>
+        <v>5.999999999994543E-2</v>
+      </c>
+      <c r="E9" s="35">
+        <f>E8-IncomeStatement!E3</f>
+        <v>3.999999999996362E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="36" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="37">
+        <f t="shared" ref="B12:E16" si="0">B3/B$8</f>
+        <v>0.52117676895764653</v>
+      </c>
+      <c r="C12" s="37">
+        <f t="shared" si="0"/>
+        <v>0.52334985650926169</v>
+      </c>
+      <c r="D12" s="37">
+        <f t="shared" si="0"/>
+        <v>0.51444643313730509</v>
+      </c>
+      <c r="E12" s="37">
+        <f t="shared" si="0"/>
+        <v>0.50360403652090346</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="B13" s="37">
+        <f t="shared" si="0"/>
+        <v>0.10195282779609437</v>
+      </c>
+      <c r="C13" s="37">
+        <f t="shared" si="0"/>
+        <v>7.6702321941038348E-2</v>
+      </c>
+      <c r="D13" s="37">
+        <f t="shared" si="0"/>
+        <v>7.6706724622858616E-2</v>
+      </c>
+      <c r="E13" s="37">
+        <f t="shared" si="0"/>
+        <v>8.097068716962999E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="37">
+        <f t="shared" si="0"/>
+        <v>7.4308901851382211E-2</v>
+      </c>
+      <c r="C14" s="37">
+        <f t="shared" si="0"/>
+        <v>7.3832507174536918E-2</v>
+      </c>
+      <c r="D14" s="37">
+        <f t="shared" si="0"/>
+        <v>6.8268984914344161E-2</v>
+      </c>
+      <c r="E14" s="37">
+        <f t="shared" si="0"/>
+        <v>6.7275348390197026E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="31" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="37">
+        <f t="shared" si="0"/>
+        <v>0.10448896779102208</v>
+      </c>
+      <c r="C15" s="37">
+        <f t="shared" si="0"/>
+        <v>0.10383511609705191</v>
+      </c>
+      <c r="D15" s="37">
+        <f t="shared" si="0"/>
+        <v>9.4604960368192284E-2</v>
+      </c>
+      <c r="E15" s="37">
+        <f t="shared" si="0"/>
+        <v>8.5776069197501206E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="B16" s="37">
+        <f t="shared" si="0"/>
+        <v>0.19807253360385493</v>
+      </c>
+      <c r="C16" s="37">
+        <f t="shared" si="0"/>
+        <v>0.22228019827811113</v>
+      </c>
+      <c r="D16" s="37">
+        <f t="shared" si="0"/>
+        <v>0.24597289695729996</v>
+      </c>
+      <c r="E16" s="37">
+        <f t="shared" si="0"/>
+        <v>0.26237385872176838</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="36" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" s="37">
+        <f t="shared" ref="C19:E23" si="1">C3/B3-1</f>
+        <v>-2.3844282238442815E-2</v>
+      </c>
+      <c r="D19" s="37">
+        <f t="shared" si="1"/>
+        <v>2.9910269192421346E-3</v>
+      </c>
+      <c r="E19" s="37">
+        <f t="shared" si="1"/>
+        <v>4.1749502982107334E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="C20" s="37">
+        <f t="shared" si="1"/>
+        <v>-0.26865671641791056</v>
+      </c>
+      <c r="D20" s="37">
+        <f t="shared" si="1"/>
+        <v>2.0408163265306145E-2</v>
+      </c>
+      <c r="E20" s="37">
+        <f t="shared" si="1"/>
+        <v>0.12333333333333352</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" s="37">
+        <f t="shared" si="1"/>
+        <v>-3.4129692832764458E-2</v>
+      </c>
+      <c r="D21" s="37">
+        <f t="shared" si="1"/>
+        <v>-5.6537102473498302E-2</v>
+      </c>
+      <c r="E21" s="37">
+        <f t="shared" si="1"/>
+        <v>4.8689138576779145E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="31" t="s">
+        <v>172</v>
+      </c>
+      <c r="C22" s="37">
+        <f t="shared" si="1"/>
+        <v>-3.3980582524271941E-2</v>
+      </c>
+      <c r="D22" s="37">
+        <f t="shared" si="1"/>
+        <v>-7.0351758793969821E-2</v>
+      </c>
+      <c r="E22" s="37">
+        <f t="shared" si="1"/>
+        <v>-3.5135135135135109E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="C23" s="37">
+        <f t="shared" si="1"/>
+        <v>9.090909090909105E-2</v>
+      </c>
+      <c r="D23" s="37">
+        <f t="shared" si="1"/>
+        <v>0.12910798122065725</v>
+      </c>
+      <c r="E23" s="37">
+        <f t="shared" si="1"/>
+        <v>0.13513513513513509</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="36" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="31" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="31" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="31" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="31" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="31" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="31" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="31" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="38" t="s">
+        <v>188</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4059,33 +4585,33 @@
     <col min="2" max="10" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="B5" s="14">
         <v>1.43</v>
@@ -4099,7 +4625,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="B6" s="14">
         <v>1.77</v>
@@ -4113,7 +4639,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="B7" s="14">
         <v>2.67</v>
@@ -4127,7 +4653,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="B8" s="14">
         <v>1.94</v>
@@ -4141,7 +4667,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="B10" s="12">
         <v>111.2</v>
@@ -4149,7 +4675,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B11" s="12">
         <v>95.4</v>
@@ -4157,7 +4683,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="B12" s="6">
         <f>B10/B11-1</f>
@@ -4166,15 +4692,15 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="B15" s="14">
         <v>1.89</v>
@@ -4182,37 +4708,37 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>